<commit_message>
Mejoras a la api
</commit_message>
<xml_diff>
--- a/cotemar/CheckListCotemar.xlsx
+++ b/cotemar/CheckListCotemar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karinabanda/Desktop/Proyectos/Reportes/Reportes Diarios/proyecto/cotemar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88296738-7DF1-3A47-8BED-C8522701C558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F812EE64-A5EF-8B45-A52B-C3B874FB1288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
   <si>
     <t>Min</t>
   </si>
@@ -45,15 +45,6 @@
     <t>VPC Name</t>
   </si>
   <si>
-    <t>VPN In (MB)</t>
-  </si>
-  <si>
-    <t>VPN Out (MB)</t>
-  </si>
-  <si>
-    <t>VPN State</t>
-  </si>
-  <si>
     <t>La revisión realizada se basa en los siguientes criterios:
 * Status Check: Verificación del estado de la vpc se encuentra en "OK".
 Recomendación: No depender únicamente de los comentarios anexados; se sugiere realizar una revisión adicional para mayor precisión.</t>
@@ -69,6 +60,18 @@
   </si>
   <si>
     <t>Tiempo de espera</t>
+  </si>
+  <si>
+    <t>4xx Errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5xx Errors </t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Latency</t>
   </si>
 </sst>
 </file>
@@ -311,6 +314,30 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -356,32 +383,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -628,83 +631,83 @@
   <sheetData>
     <row r="1" spans="2:17" ht="15.75" customHeight="1"/>
     <row r="2" spans="2:17" ht="27" customHeight="1">
-      <c r="B2" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
+      <c r="B2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
     </row>
     <row r="3" spans="2:17" ht="27" customHeight="1">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
+      <c r="C3" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="11"/>
+      <c r="N3" s="11"/>
     </row>
     <row r="4" spans="2:17" ht="22" customHeight="1">
-      <c r="B4" s="21"/>
-      <c r="C4" s="23" t="s">
+      <c r="B4" s="27"/>
+      <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="I4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="J4" s="23" t="s">
+      <c r="J4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L4" s="23" t="s">
+      <c r="L4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="M4" s="23" t="s">
+      <c r="M4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="N4" s="23" t="s">
+      <c r="N4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
@@ -754,181 +757,181 @@
     </row>
     <row r="8" spans="2:17" ht="15.75" customHeight="1"/>
     <row r="9" spans="2:17" ht="27" customHeight="1">
-      <c r="B9" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
+      <c r="B9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
       <c r="P9" s="2"/>
       <c r="Q9" s="1"/>
     </row>
     <row r="10" spans="2:17" ht="18" customHeight="1">
-      <c r="B10" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="H10" s="7" t="s">
+      <c r="B10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="H10" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="9"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="17"/>
     </row>
     <row r="11" spans="2:17" ht="15.75" customHeight="1">
-      <c r="B11" s="27"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="H11" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="12"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="H11" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="20"/>
     </row>
     <row r="12" spans="2:17" ht="22" customHeight="1">
-      <c r="B12" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="15"/>
+      <c r="B12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="23"/>
     </row>
     <row r="13" spans="2:17" ht="15.75" customHeight="1">
-      <c r="H13" s="13"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="14"/>
-      <c r="N13" s="15"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="23"/>
     </row>
     <row r="14" spans="2:17" ht="17" customHeight="1">
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
-      <c r="N14" s="15"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="23"/>
       <c r="Q14" s="2"/>
     </row>
     <row r="15" spans="2:17" ht="25" customHeight="1">
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="9"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="15"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="23"/>
       <c r="Q15" s="2"/>
     </row>
     <row r="16" spans="2:17" ht="15.75" customHeight="1">
-      <c r="B16" s="4"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="6"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="15"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="14"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="23"/>
     </row>
     <row r="17" spans="2:14" ht="15" customHeight="1">
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="15"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="23"/>
     </row>
     <row r="18" spans="2:14" ht="14" customHeight="1">
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-      <c r="N18" s="15"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="23"/>
     </row>
     <row r="19" spans="2:14" ht="15.75" customHeight="1">
-      <c r="H19" s="13"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="14"/>
-      <c r="N19" s="15"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="23"/>
     </row>
     <row r="20" spans="2:14" ht="15" customHeight="1">
-      <c r="H20" s="13"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="15"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="23"/>
     </row>
     <row r="21" spans="2:14" ht="15" customHeight="1">
-      <c r="H21" s="13"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="15"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="23"/>
     </row>
     <row r="22" spans="2:14" ht="15" customHeight="1">
-      <c r="H22" s="16"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="18"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="25"/>
+      <c r="M22" s="25"/>
+      <c r="N22" s="26"/>
     </row>
     <row r="23" spans="2:14" ht="17" customHeight="1"/>
     <row r="25" spans="2:14" ht="15.75" customHeight="1"/>
@@ -1907,11 +1910,6 @@
     <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C11:F11"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="L3:N3"/>
@@ -1924,6 +1922,11 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:F11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>